<commit_message>
docs(proyecto): agregar README y alinear ficha y conclusiones con el modelo final
</commit_message>
<xml_diff>
--- a/FO-IV-159-GRUPO-F.xlsx
+++ b/FO-IV-159-GRUPO-F.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juans\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juans\IdeaProjects\fuel-consumption-prediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2E9936-BFED-4A7F-BBD8-3F799701E20E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19067523-BA69-4EFF-86AE-491481052701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -905,15 +905,9 @@
     <t>Analisis de Datos / Big Data</t>
   </si>
   <si>
-    <t>¿En qué medida la distancia recorrida, el tipo de barco y el tipo de combustible explican la variación en el consumo de combustible de las embarcaciones mediante un modelo de regresión lineal múltiple?</t>
-  </si>
-  <si>
     <t>Este proyecto se justifica por la necesidad de comprender las variaciones en el consumo de combustible de las embarcaciones y aportar información útil para su planificación operativa. Analizar los factores relacionados con este consumo puede apoyar la estimación de las necesidades de combustible, la elaboración de presupuestos y la identificación de oportunidades para utilizar los recursos de manera más eficiente.
 La regresión lineal múltiple permite estudiar conjuntamente las dos variables independientes seleccionadas y estimar su relación con el consumo de combustible. Su aplicación, acompañada de la evaluación de los supuestos estadísticos, permite valorar el alcance y las limitaciones de los resultados obtenidos.
 Desde el ámbito académico, el proyecto fortalece las competencias en preparación y exploración de datos, construcción de modelos e interpretación de resultados. Asimismo, vincula el análisis estadístico con una situación de interés económico y ambiental, al estudiar el uso de combustible en las operaciones marítimas.</t>
-  </si>
-  <si>
-    <t>Analizar la relación entre la distancia recorrida, el tipo de embarcación y el tipo de combustible y el consumo de combustible, mediante un modelo de regresión lineal múltiple que aporte información para la planificación del consumo.</t>
   </si>
   <si>
     <t>*Describir las características de las embarcaciones y el comportamiento de las variables incluidas en    la base de datos.
@@ -931,11 +925,6 @@
 Interpretación: análisis de los coeficientes, los valores p y el coeficiente de determinación ajustado para valorar las relaciones encontradas, el ajuste del modelo y sus limitaciones.</t>
   </si>
   <si>
-    <t>Se realizó el análisis exploratorio de la distancia recorrida, el consumo de combustible y las emisiones de CO₂ de las embarcaciones mediante estadísticas descriptivas, gráficos de dispersión y una matriz de correlación. Este análisis permitió examinar las relaciones entre las tres variables y fundamentar su selección para el ejercicio de regresión lineal múltiple.
-Se construyó un modelo con las emisiones de CO₂ como variable dependiente y la distancia recorrida y el consumo de combustible como variables independientes. El ejercicio permitió analizar su relación conjunta con las emisiones y desarrollar la interpretación de los coeficientes y de las medidas de ajuste del modelo.
-Como resultado académico, se fortalecieron las competencias en procesamiento de datos, modelación estadística e interpretación crítica de resultados, reconociendo que una asociación estadística no demuestra por sí sola una relación causal.</t>
-  </si>
-  <si>
     <t>Cuaderno de Google Colab con el código del análisis exploratorio y del modelo de regresión lineal múltiple.
 Tablas de estadísticas descriptivas y matriz de correlación de las variables estudiadas.
 Gráficos de dispersión y gráficos de diagnóstico del modelo.
@@ -954,6 +943,18 @@
   <si>
     <t>La planificación del combustible en las embarcaciones requiere comprender por qué su consumo varía entre los registros de operación. Utilizar únicamente promedios generales puede ocultar diferencias relevantes y limitar la estimación de las necesidades de combustible y de los costos asociados a cada recorrido.
 En este estudio se busca determinar en qué medida las variables explicativas seleccionadas permiten comprender la variación del consumo de combustible en las embarcaciones analizadas. Para ello, se empleará un modelo de regresión lineal múltiple que permita evaluar la relación de cada variable con el consumo, manteniendo constante la otra, y examinar el cumplimiento de los supuestos estadísticos. El análisis busca aportar información que sirva de apoyo para una mejor planificación del combustible.</t>
+  </si>
+  <si>
+    <t>Se realizó el análisis exploratorio de las variables de la base de datos (distancia recorrida, consumo de combustible, tipo de barco, tipo de combustible, eficiencia del motor, entre otras) mediante estadísticas descriptivas, gráficos de dispersión y una matriz de correlación. Este análisis permitió examinar las relaciones entre las variables y fundamentar la selección de la distancia recorrida y el tipo de barco como variables independientes del modelo de regresión lineal múltiple.
+Se construyó un modelo con el consumo de combustible como variable dependiente y la distancia recorrida y el tipo de barco como variables independientes. El modelo inicial explicó el 94.3 % de la variación del consumo, pero el diagnóstico de residuos mostró falta de linealidad, heterocedasticidad y desviaciones de la normalidad. Por esto se aplicó una transformación logarítmica, con la que el R² ajustado subió a 0.974, y se usaron errores estándar robustos HC3 para que la inferencia fuera confiable. Los residuos resultaron independientes (Durbin-Watson ≈ 2.06) y no se encontraron problemas de multicolinealidad.
+El coeficiente de la distancia fue cercano a 1, lo que indica que el consumo crece de forma proporcional a la distancia recorrida. Para una misma distancia, y frente a un Fishing Trawler, un Tanker Ship consume cerca de un 59 % más, un Oil Service Boat un 20 % más y un Surfer Boat un 41 % menos. El tipo de combustible casi no mejoró el ajuste del modelo, y el clima, la ruta, el mes y la eficiencia del motor no resultaron significativos.
+Como resultado académico, se fortalecieron las competencias en procesamiento de datos, modelación estadística e interpretación crítica de resultados, reconociendo que una asociación estadística no demuestra por sí sola una relación causal.</t>
+  </si>
+  <si>
+    <t>¿En qué medida la distancia recorrida y el tipo de barco explican la variación en el consumo de combustible de las embarcaciones mediante un modelo de regresión lineal múltiple?</t>
+  </si>
+  <si>
+    <t>Analizar la relación entre la distancia recorrida, el tipo de embarcación y el consumo de combustible, mediante un modelo de regresión lineal múltiple que aporte información para la planificación del consumo.</t>
   </si>
 </sst>
 </file>
@@ -2646,7 +2647,7 @@
       </c>
       <c r="C7" s="54"/>
       <c r="D7" s="56" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="E7" s="57"/>
       <c r="F7" s="58"/>
@@ -2730,7 +2731,7 @@
       </c>
       <c r="C13" s="54"/>
       <c r="D13" s="69" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E13" s="53"/>
       <c r="F13" s="54"/>
@@ -2783,7 +2784,7 @@
       </c>
       <c r="C17" s="54"/>
       <c r="D17" s="56" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E17" s="57"/>
       <c r="F17" s="58"/>
@@ -2797,7 +2798,7 @@
       </c>
       <c r="C18" s="54"/>
       <c r="D18" s="56" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="E18" s="57"/>
       <c r="F18" s="58"/>
@@ -2811,7 +2812,7 @@
       </c>
       <c r="C19" s="54"/>
       <c r="D19" s="56" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E19" s="57"/>
       <c r="F19" s="58"/>
@@ -2835,7 +2836,7 @@
       </c>
       <c r="C21" s="54"/>
       <c r="D21" s="56" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="E21" s="57"/>
       <c r="F21" s="58"/>
@@ -2849,7 +2850,7 @@
       </c>
       <c r="C22" s="54"/>
       <c r="D22" s="56" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E22" s="57"/>
       <c r="F22" s="58"/>
@@ -2863,7 +2864,7 @@
       </c>
       <c r="C23" s="54"/>
       <c r="D23" s="56" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E23" s="57"/>
       <c r="F23" s="58"/>
@@ -2879,7 +2880,7 @@
       <c r="E24" s="53"/>
       <c r="F24" s="54"/>
     </row>
-    <row r="25" spans="1:7" ht="219" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="389.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>18</v>
       </c>
@@ -2888,7 +2889,7 @@
       </c>
       <c r="C25" s="54"/>
       <c r="D25" s="56" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E25" s="57"/>
       <c r="F25" s="58"/>
@@ -2903,7 +2904,7 @@
       </c>
       <c r="C26" s="54"/>
       <c r="D26" s="56" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E26" s="57"/>
       <c r="F26" s="58"/>
@@ -2950,7 +2951,7 @@
       </c>
       <c r="C30" s="54"/>
       <c r="D30" s="61" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E30" s="57"/>
       <c r="F30" s="58"/>

</xml_diff>

<commit_message>
docs(proyecto): Actualización del README y ipynb
</commit_message>
<xml_diff>
--- a/FO-IV-159-GRUPO-F.xlsx
+++ b/FO-IV-159-GRUPO-F.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juans\IdeaProjects\fuel-consumption-prediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19067523-BA69-4EFF-86AE-491481052701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D55FF4-0A96-4069-B304-4A4DB2EBC3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -931,10 +931,6 @@
 Informe del taller con la metodología, la interpretación de los resultados y las conclusiones.</t>
   </si>
   <si>
-    <t>jose-llanos. (s. f.). TecnicasAnalisisEstadistico: Unidad 4 [Repositorio de GitHub]. GitHub. https://github.com/jose-llanos/TecnicasAnalisisEstadistico/tree/main/unidad-4     
-Corporación Universitaria del Huila. (s. f.). Técnicas de análisis estadístico: Unidad de aprendizaje 4, regresión lineal [Material de curso]. CORHUILA Digital. https://virtual.corhuila.edu.co/uh/course/view.php?id=5111</t>
-  </si>
-  <si>
     <t>BigData y Analítica de datos</t>
   </si>
   <si>
@@ -955,6 +951,10 @@
   </si>
   <si>
     <t>Analizar la relación entre la distancia recorrida, el tipo de embarcación y el consumo de combustible, mediante un modelo de regresión lineal múltiple que aporte información para la planificación del consumo.</t>
+  </si>
+  <si>
+    <t>jose-llanos. (s. f.). TecnicasAnalisisEstadistico: Unidad 4 [Repositorio de GitHub]. GitHub. https://github.com/jose-llanos/TecnicasAnalisisEstadistico/tree/main/unidad-4     
+Llanos Mosquera, J. M. (s. f.). *TAE-Unidad de aprendizaje 4: Regresión Lineal*. Recuperado 10 de octubre de 2026, de https://virtual.corhuila.edu.co/uh/mod/resource/view.php?id=124121</t>
   </si>
 </sst>
 </file>
@@ -1663,13 +1663,32 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1680,22 +1699,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1707,33 +1714,26 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2518,27 +2518,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70"/>
-      <c r="B1" s="71"/>
-      <c r="C1" s="76" t="s">
+      <c r="A1" s="52"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="54"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="60"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="72"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="77" t="s">
+      <c r="A2" s="54"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="71"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="53"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2555,12 +2555,12 @@
       <c r="T2" s="1"/>
     </row>
     <row r="3" spans="1:20" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="72"/>
-      <c r="B3" s="73"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="75"/>
+      <c r="A3" s="54"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="57"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -2577,8 +2577,8 @@
       <c r="T3" s="1"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="74"/>
-      <c r="B4" s="75"/>
+      <c r="A4" s="56"/>
+      <c r="B4" s="57"/>
       <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
@@ -2607,12 +2607,12 @@
       <c r="T4" s="1"/>
     </row>
     <row r="5" spans="1:20" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="80"/>
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="54"/>
+      <c r="A5" s="64"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="60"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -2629,350 +2629,350 @@
       <c r="T5" s="1"/>
     </row>
     <row r="6" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="81" t="s">
+      <c r="A6" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="60"/>
     </row>
     <row r="7" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>1</v>
       </c>
-      <c r="B7" s="63" t="s">
+      <c r="B7" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="54"/>
-      <c r="D7" s="56" t="s">
-        <v>289</v>
-      </c>
-      <c r="E7" s="57"/>
-      <c r="F7" s="58"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="67" t="s">
+        <v>288</v>
+      </c>
+      <c r="E7" s="68"/>
+      <c r="F7" s="69"/>
     </row>
     <row r="8" spans="1:20" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>2</v>
       </c>
-      <c r="B8" s="63" t="s">
+      <c r="B8" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="54"/>
-      <c r="D8" s="56" t="s">
+      <c r="C8" s="60"/>
+      <c r="D8" s="67" t="s">
         <v>281</v>
       </c>
-      <c r="E8" s="57"/>
-      <c r="F8" s="58"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="69"/>
     </row>
     <row r="9" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>3</v>
       </c>
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="69" t="s">
+      <c r="C9" s="60"/>
+      <c r="D9" s="70" t="s">
         <v>282</v>
       </c>
-      <c r="E9" s="53"/>
-      <c r="F9" s="54"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="60"/>
     </row>
     <row r="10" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>5</v>
       </c>
-      <c r="B10" s="63" t="s">
+      <c r="B10" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="54"/>
-      <c r="D10" s="68">
+      <c r="C10" s="60"/>
+      <c r="D10" s="71">
         <v>46300</v>
       </c>
-      <c r="E10" s="65"/>
-      <c r="F10" s="66"/>
+      <c r="E10" s="72"/>
+      <c r="F10" s="73"/>
     </row>
     <row r="11" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>6</v>
       </c>
-      <c r="B11" s="63" t="s">
+      <c r="B11" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="54"/>
-      <c r="D11" s="68">
+      <c r="C11" s="60"/>
+      <c r="D11" s="71">
         <v>46305</v>
       </c>
-      <c r="E11" s="65"/>
-      <c r="F11" s="66"/>
+      <c r="E11" s="72"/>
+      <c r="F11" s="73"/>
     </row>
     <row r="12" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>8</v>
       </c>
-      <c r="B12" s="63" t="s">
+      <c r="B12" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="54"/>
-      <c r="D12" s="67" t="s">
+      <c r="C12" s="60"/>
+      <c r="D12" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="53"/>
-      <c r="F12" s="54"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="60"/>
     </row>
     <row r="13" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>9</v>
       </c>
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="66" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="54"/>
-      <c r="D13" s="69" t="s">
-        <v>288</v>
-      </c>
-      <c r="E13" s="53"/>
-      <c r="F13" s="54"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="70" t="s">
+        <v>287</v>
+      </c>
+      <c r="E13" s="59"/>
+      <c r="F13" s="60"/>
     </row>
     <row r="14" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>10</v>
       </c>
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="64">
+      <c r="C14" s="60"/>
+      <c r="D14" s="75">
         <v>1</v>
       </c>
-      <c r="E14" s="65"/>
-      <c r="F14" s="66"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="73"/>
     </row>
     <row r="15" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>11</v>
       </c>
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="54"/>
-      <c r="D15" s="67" t="s">
+      <c r="C15" s="60"/>
+      <c r="D15" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="53"/>
-      <c r="F15" s="54"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="60"/>
       <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="59" t="s">
+      <c r="A16" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="54"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="60"/>
     </row>
     <row r="17" spans="1:7" ht="199.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>12</v>
       </c>
-      <c r="B17" s="63" t="s">
+      <c r="B17" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="56" t="s">
-        <v>290</v>
-      </c>
-      <c r="E17" s="57"/>
-      <c r="F17" s="58"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="67" t="s">
+        <v>289</v>
+      </c>
+      <c r="E17" s="68"/>
+      <c r="F17" s="69"/>
     </row>
     <row r="18" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>13</v>
       </c>
-      <c r="B18" s="63" t="s">
+      <c r="B18" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="54"/>
-      <c r="D18" s="56" t="s">
-        <v>292</v>
-      </c>
-      <c r="E18" s="57"/>
-      <c r="F18" s="58"/>
+      <c r="C18" s="60"/>
+      <c r="D18" s="67" t="s">
+        <v>291</v>
+      </c>
+      <c r="E18" s="68"/>
+      <c r="F18" s="69"/>
     </row>
     <row r="19" spans="1:7" ht="258.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>14</v>
       </c>
-      <c r="B19" s="63" t="s">
+      <c r="B19" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="54"/>
-      <c r="D19" s="56" t="s">
+      <c r="C19" s="60"/>
+      <c r="D19" s="67" t="s">
         <v>283</v>
       </c>
-      <c r="E19" s="57"/>
-      <c r="F19" s="58"/>
+      <c r="E19" s="68"/>
+      <c r="F19" s="69"/>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="59" t="s">
+      <c r="A20" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="53"/>
-      <c r="C20" s="53"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="54"/>
+      <c r="B20" s="59"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="60"/>
     </row>
     <row r="21" spans="1:7" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>15</v>
       </c>
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="54"/>
-      <c r="D21" s="56" t="s">
-        <v>293</v>
-      </c>
-      <c r="E21" s="57"/>
-      <c r="F21" s="58"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="67" t="s">
+        <v>292</v>
+      </c>
+      <c r="E21" s="68"/>
+      <c r="F21" s="69"/>
     </row>
     <row r="22" spans="1:7" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>16</v>
       </c>
-      <c r="B22" s="63" t="s">
+      <c r="B22" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="54"/>
-      <c r="D22" s="56" t="s">
+      <c r="C22" s="60"/>
+      <c r="D22" s="67" t="s">
         <v>284</v>
       </c>
-      <c r="E22" s="57"/>
-      <c r="F22" s="58"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="69"/>
     </row>
     <row r="23" spans="1:7" ht="369.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>17</v>
       </c>
-      <c r="B23" s="63" t="s">
+      <c r="B23" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="54"/>
-      <c r="D23" s="56" t="s">
+      <c r="C23" s="60"/>
+      <c r="D23" s="67" t="s">
         <v>285</v>
       </c>
-      <c r="E23" s="57"/>
-      <c r="F23" s="58"/>
+      <c r="E23" s="68"/>
+      <c r="F23" s="69"/>
       <c r="G23" s="5"/>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="59" t="s">
+      <c r="A24" s="76" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="53"/>
-      <c r="C24" s="53"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="53"/>
-      <c r="F24" s="54"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="60"/>
     </row>
     <row r="25" spans="1:7" ht="389.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>18</v>
       </c>
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="54"/>
-      <c r="D25" s="56" t="s">
-        <v>291</v>
-      </c>
-      <c r="E25" s="57"/>
-      <c r="F25" s="58"/>
+      <c r="C25" s="60"/>
+      <c r="D25" s="67" t="s">
+        <v>290</v>
+      </c>
+      <c r="E25" s="68"/>
+      <c r="F25" s="69"/>
       <c r="G25" s="5"/>
     </row>
     <row r="26" spans="1:7" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>19</v>
       </c>
-      <c r="B26" s="62" t="s">
+      <c r="B26" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="56" t="s">
+      <c r="C26" s="60"/>
+      <c r="D26" s="67" t="s">
         <v>286</v>
       </c>
-      <c r="E26" s="57"/>
-      <c r="F26" s="58"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="69"/>
       <c r="G26" s="5"/>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="59" t="s">
+      <c r="A27" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="53"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="54"/>
+      <c r="B27" s="59"/>
+      <c r="C27" s="59"/>
+      <c r="D27" s="59"/>
+      <c r="E27" s="59"/>
+      <c r="F27" s="60"/>
     </row>
     <row r="28" spans="1:7" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>20</v>
       </c>
-      <c r="B28" s="63" t="s">
+      <c r="B28" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="54"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="54"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="59"/>
+      <c r="F28" s="60"/>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="53"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="54"/>
+      <c r="B29" s="59"/>
+      <c r="C29" s="59"/>
+      <c r="D29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="60"/>
     </row>
     <row r="30" spans="1:7" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>21</v>
       </c>
-      <c r="B30" s="63" t="s">
+      <c r="B30" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="54"/>
-      <c r="D30" s="61" t="s">
-        <v>287</v>
-      </c>
-      <c r="E30" s="57"/>
-      <c r="F30" s="58"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="80" t="s">
+        <v>293</v>
+      </c>
+      <c r="E30" s="68"/>
+      <c r="F30" s="69"/>
     </row>
     <row r="31" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="A31" s="77"/>
+      <c r="B31" s="59"/>
+      <c r="C31" s="59"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="60"/>
     </row>
     <row r="32" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="78" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="53"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="54"/>
+      <c r="B32" s="59"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="60"/>
     </row>
     <row r="33" spans="6:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F33" s="5"/>
@@ -4344,40 +4344,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="C2:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B25:C25"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="D19:F19"/>
@@ -4394,6 +4360,40 @@
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="C2:F3"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="38" orientation="landscape"/>

</xml_diff>